<commit_message>
Tasa de Fallo Calculada
</commit_message>
<xml_diff>
--- a/Optimization/Resultados.xlsx
+++ b/Optimization/Resultados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oso_e\maestria\Maestria\Optimization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA771241-61D8-4D11-8B40-CE8387A4C2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912279D7-E92C-446B-A197-D9D24D17F680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,28 +25,59 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Fecha</t>
   </si>
   <si>
     <t>Tipo De Prueba</t>
+  </si>
+  <si>
+    <t>Plataforma</t>
+  </si>
+  <si>
+    <t>Usuario</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>Grupos</t>
+  </si>
+  <si>
+    <t>MultiplesGrupos</t>
+  </si>
+  <si>
+    <t>Confianza</t>
+  </si>
+  <si>
+    <t>Gatito</t>
+  </si>
+  <si>
+    <t>Joya</t>
+  </si>
+  <si>
+    <t>Quique</t>
+  </si>
+  <si>
+    <t>NoQuique</t>
+  </si>
+  <si>
+    <t>Fallo</t>
+  </si>
+  <si>
+    <t>fallo</t>
+  </si>
+  <si>
+    <t>Paso</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -74,9 +105,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,21 +389,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46006</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>46006</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46006</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>